<commit_message>
Invoice Refresh workbook: link to each case's result in run R417, not the case
The column now points at /tests/view/<test_id> - the recorded result, its comment
and its history inside the run - instead of the case definition. Test ids are read
live from the run, since they are per-run and cannot be derived from the C-id.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FWbxRKg4riKCp3gpbbwYzA
</commit_message>
<xml_diff>
--- a/build/invoice-ui-refresh/execution-2026-09-07/Invoice-UI-Refresh_Failed-and-Blocked-Cases_2026-09-08.xlsx
+++ b/build/invoice-ui-refresh/execution-2026-09-07/Invoice-UI-Refresh_Failed-and-Blocked-Cases_2026-09-08.xlsx
@@ -720,7 +720,7 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>TestRail link</t>
+          <t>Result in test run R417</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44917</t>
+          <t>https://shopview.testrail.io/index.php?/tests/view/2724080</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44926</t>
+          <t>https://shopview.testrail.io/index.php?/tests/view/2724089</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44935</t>
+          <t>https://shopview.testrail.io/index.php?/tests/view/2724098</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44952</t>
+          <t>https://shopview.testrail.io/index.php?/tests/view/2724115</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44970</t>
+          <t>https://shopview.testrail.io/index.php?/tests/view/2724133</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44974</t>
+          <t>https://shopview.testrail.io/index.php?/tests/view/2724137</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>TestRail link</t>
+          <t>Result in test run R417</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44902</t>
+          <t>https://shopview.testrail.io/index.php?/tests/view/2724065</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44907</t>
+          <t>https://shopview.testrail.io/index.php?/tests/view/2724070</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/44916</t>
+          <t>https://shopview.testrail.io/index.php?/tests/view/2724079</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/45275</t>
+          <t>https://shopview.testrail.io/index.php?/tests/view/2867755</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">

</xml_diff>

<commit_message>
C44952 passes: Chris amended S8-R9, the Remaining Balance row was never a requirement
Chris Ward ruled on SV-9803 that the paid banner's Remaining Balance row has never
existed in production - settled by the matching sha256 on the portal banner chunk
across production and staging - and amended the spec to v64. Verified at source:
the phrase now appears only in the Story 8 context note and the change-log row,
both saying no such row exists.

C44952: clause 4 deleted, clauses renumbered, the three-outcome block removed, and
the provenance re-stamped to spec v64 / build v26.35.9-9812433. Re-scored Passed in
R417, which now reads 111 Passed, 5 Failed, 4 Blocked, 0 untested. The build never
changed.

Workbook and release-readiness record updated to match.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FWbxRKg4riKCp3gpbbwYzA
</commit_message>
<xml_diff>
--- a/build/invoice-ui-refresh/execution-2026-09-07/Invoice-UI-Refresh_Failed-and-Blocked-Cases_2026-09-08.xlsx
+++ b/build/invoice-ui-refresh/execution-2026-09-07/Invoice-UI-Refresh_Failed-and-Blocked-Cases_2026-09-08.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Blocked" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Failed'!$A$1:$H$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Failed'!$A$1:$H$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -588,90 +588,94 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr"/>
-      <c r="B9" s="2" t="inlineStr"/>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Last updated</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>8 September 2026 - C44952 re-scored Passed after the spec was amended</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Cases in the suite</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>120</t>
-        </is>
-      </c>
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Cases in the suite</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>120</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>6   - see the Failed tab</t>
+          <t>111</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Failed</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>4   - see the Blocked tab</t>
+          <t>5   - see the Failed tab</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>4   - see the Blocked tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
           <t>Untested</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr"/>
-      <c r="B15" s="2" t="inlineStr"/>
-    </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Read this first</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>FAILED means the build does not do what the documents require. Every one of these except C44952 already has a ticket, so there is nothing for you to raise.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr"/>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>BLOCKED means the case could not be run at all. Three of the four are still worth keeping - they need a decision or a piece of test data from you, and each row says exactly what and who. The fourth is an empty case that only its author can fix.</t>
+          <t>FAILED means the build does not do what the documents require. Every one of these already has a ticket, so there is nothing for you to raise.</t>
         </is>
       </c>
     </row>
@@ -679,7 +683,23 @@
       <c r="A18" s="3" t="inlineStr"/>
       <c r="B18" s="2" t="inlineStr">
         <is>
+          <t>BLOCKED means the case could not be run at all. Three of the four are still worth keeping - they need a decision or a piece of test data from you, and each row says exactly what and who. The fourth is an empty case that only its author can fix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr"/>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
           <t>Two tickets - SV-9642 and SV-9773 - moved to QA Complete AFTER this run. Both cases were still failing on the build tested, so both need re-running on the next staging build.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>C44952 was Failed on 7 September and is now PASSED. It failed only on a "Remaining Balance" row that the specification asked for. Chris Ward established that row has never existed in production and amended S8-R9 (spec v64, SV-9803). The clause is gone from the case; the build never changed.</t>
         </is>
       </c>
     </row>
@@ -694,7 +714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -878,154 +898,116 @@
     <row r="5" ht="118" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>C44952</t>
+          <t>C44970</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Each banner payment shows its labeled fields and conditional fees/marker</t>
+          <t>Credit Invoice shows the disclaimer and standard signature area</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/tests/view/2724115</t>
+          <t>https://shopview.testrail.io/index.php?/tests/view/2724133</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>SV-9790</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>NO OPEN TICKET</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr"/>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>https://shopview.atlassian.net/browse/SV-9790</t>
+        </is>
+      </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>In the customer portal, the paid-invoice banner never shows a "Remaining Balance" row, even when money is still owed after a payment. Everything else in the banner is correct.</t>
+          <t>A credit note created on its own prints no disclaimer text at the bottom. One created from an invoice does print it. Both should.</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>NO OPEN TICKET. This was raised as SV-9803 and you closed it as OBSOLETE on 7 September. The case still fails as written. Either the rule should be dropped from the specification, or a ticket has to be raised - your call. Nobody should raise one without you.</t>
+          <t>Nothing for you to do. The ticket is Open and waiting on development. Re-run this case once it ships.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="118" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>C44970</t>
+          <t>C44974</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Credit Invoice shows the disclaimer and standard signature area</t>
+          <t>Typography uses Inter with the specified weights</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/tests/view/2724133</t>
+          <t>https://shopview.testrail.io/index.php?/tests/view/2724137</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>SV-9790</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>SV-9761</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>TESTING STAGE</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>https://shopview.atlassian.net/browse/SV-9790</t>
+          <t>https://shopview.atlassian.net/browse/SV-9761</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>A credit note created on its own prints no disclaimer text at the bottom. One created from an invoice does print it. Both should.</t>
+          <t>The printed documents use the wrong typeface. Every PDF checked embeds DejaVu Sans, not the Inter font the design asks for.</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Nothing for you to do. The ticket is Open and waiting on development. Re-run this case once it ships.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="118" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>C44974</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Typography uses Inter with the specified weights</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/tests/view/2724137</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>SV-9761</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>TESTING STAGE</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>https://shopview.atlassian.net/browse/SV-9761</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>The printed documents use the wrong typeface. Every PDF checked embeds DejaVu Sans, not the Inter font the design asks for.</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
           <t>Nothing for you to do here, but note the second ticket: SV-9781 records that the LIVE PDF server still has the old font too, so this will still be wrong after release unless that is also done.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="44" customHeight="1">
-      <c r="A9" s="9" t="inlineStr">
+    <row r="8" ht="44" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Also on C44974:</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>SV-9781</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>Board Backlog</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>https://shopview.atlassian.net/browse/SV-9781</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>The LIVE PDF server still carries the old font image, so the wrong typeface will still be there after release even once staging is fixed.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H7"/>
+  <autoFilter ref="A1:H6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
C45275 is not empty: it uses separated steps, and six tools cannot read them
The 7 September triage read custom_steps and custom_expected, which are both null
on a separated-steps case, and reported C45275 as empty and unfixable. It has five
steps and a full expected-results block. No defect, no ticket needed - it simply
needs running.

Corrected the run comment, RESULTS.json and the workbook row. Recorded as L37,
including the measured finding that no tool in build/testing-tools reads
custom_steps_separated, so six of them mis-handle every such case - snapshot_case_bodies.py
worst of all, since Rule 87 depends on it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FWbxRKg4riKCp3gpbbwYzA
</commit_message>
<xml_diff>
--- a/build/invoice-ui-refresh/execution-2026-09-07/Invoice-UI-Refresh_Failed-and-Blocked-Cases_2026-09-08.xlsx
+++ b/build/invoice-ui-refresh/execution-2026-09-07/Invoice-UI-Refresh_Failed-and-Blocked-Cases_2026-09-08.xlsx
@@ -1300,14 +1300,14 @@
           <t>https://shopview.testrail.io/index.php?/tests/view/2867755</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>CANNOT SAY - the case is empty</t>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>KEEP - it is a good case that was never run</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>This case has a title and a precondition but NO steps and NO expected result recorded in TestRail. There is literally nothing written down to check, so it cannot be passed or failed by anybody. It was created by Vladimir Tomovic, and we never change his cases.</t>
+          <t>It was reported on 7 September as an empty case with nothing to check. THAT WAS WRONG. The case is written in the step-by-step format, so its content sits somewhere different from the plain Steps and Expected Result boxes, and the earlier check looked in the wrong place. It has five steps and a full set of expected results. It checks that changing only the CONTACT on a work order leaves the Authorizer alone, that changing the CUSTOMER clears the Authorizer to "None", that the picker then offers only the new customer's "Approves Work" contacts with the "No authorizer" row first, and that the new choice saves.</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
@@ -1323,20 +1323,20 @@
       <c r="H5" s="5" t="inlineStr"/>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Vladimir needs to either finish the case or retire it. Nothing else will unblock it.</t>
+          <t>Nothing to decide and no ticket needed - there is no defect here. The case simply has to be RUN. The only thing standing in the way is that the staging sign-in details are kept outside the repository for security and have been wiped from this machine, so I cannot sign in to run it.</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>VLADIMIR TOMOVIC, or you on his behalf. I am not permitted to edit his cases under any circumstances, so this one can only be cleared by him.</t>
+          <t>ME, as soon as you re-supply the staging sign-in details. Nobody else needs to do anything.</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>1. Ask Vladimir whether this case is still wanted.
-2. If YES - he fills in the Steps and the Expected Result, and tells me. I run it the same day.
-3. If NO - he retires or deletes it, and it drops out of the suite count of 120.
-4. Either way, tell me which, so the run stops showing a blocked case nobody is working on.</t>
+          <t>1. Send me the staging username and password again (they are deliberately not stored in the repository, and this machine has been cleared).
+2. I sign in, seed two customers each with an "Approves Work" contact, raise an estimate for the first, and walk the five steps.
+3. I record Passed or Failed against this case and tell you the same day.
+Note: the case belongs to Vladimir Tomovic and is flagged Automated, so its wording will not be touched - only a result recorded.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
C45275 executed and PASSED: 112 Passed, 5 Failed, 3 Blocked
Ran the case end to end through the UI on build v26.35.9-9812433. All five clauses
pass: changing only the contact leaves the Authorizer alone, changing the customer
clears it to None, the picker then offers only the new customer's Approves Work
contact with No authorizer first, and the choice saves.

Set-up was work order S2-32272, an estimate raised for Abode Trucking & Repair,
switched to Ado Truck Center - Oasis. Eight screenshots, the observations and the
run script are committed under evidence-c45275/. The case is Vladimir's and flagged
Automated, so nothing about it was edited - only a result recorded.

Also adds the ticket number and live ticket status as a fresh comment on each of the
five failed tests, since results are append-only.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FWbxRKg4riKCp3gpbbwYzA
</commit_message>
<xml_diff>
--- a/build/invoice-ui-refresh/execution-2026-09-07/Invoice-UI-Refresh_Failed-and-Blocked-Cases_2026-09-08.xlsx
+++ b/build/invoice-ui-refresh/execution-2026-09-07/Invoice-UI-Refresh_Failed-and-Blocked-Cases_2026-09-08.xlsx
@@ -623,7 +623,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>111</t>
+          <t>112</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>4   - see the Blocked tab</t>
+          <t>3   - see the Blocked tab</t>
         </is>
       </c>
     </row>
@@ -699,7 +699,7 @@
       <c r="A20" s="3" t="inlineStr"/>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>C44952 was Failed on 7 September and is now PASSED. It failed only on a "Remaining Balance" row that the specification asked for. Chris Ward established that row has never existed in production and amended S8-R9 (spec v64, SV-9803). The clause is gone from the case; the build never changed.</t>
+          <t>C45275 was reported Blocked as an empty case on 7 September. It is not empty - it uses the step-by-step format - and on 8 September it was executed in full and PASSED. C44952 was Failed on 7 September and is now PASSED. It failed only on a "Remaining Balance" row that the specification asked for. Chris Ward established that row has never existed in production and amended S8-R9 (spec v64, SV-9803). The clause is gone from the case; the build never changed.</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1284,69 +1284,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="250" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>C45275</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Changing the customer clears the Authorizer; changing only the contact does not</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/tests/view/2867755</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>KEEP - it is a good case that was never run</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>It was reported on 7 September as an empty case with nothing to check. THAT WAS WRONG. The case is written in the step-by-step format, so its content sits somewhere different from the plain Steps and Expected Result boxes, and the earlier check looked in the wrong place. It has five steps and a full set of expected results. It checks that changing only the CONTACT on a work order leaves the Authorizer alone, that changing the CUSTOMER clears the Authorizer to "None", that the picker then offers only the new customer's "Approves Work" contacts with the "No authorizer" row first, and that the new choice saves.</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="G5" s="11" t="inlineStr">
-        <is>
-          <t>NO TICKET</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr"/>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>Nothing to decide and no ticket needed - there is no defect here. The case simply has to be RUN. The only thing standing in the way is that the staging sign-in details are kept outside the repository for security and have been wiped from this machine, so I cannot sign in to run it.</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>ME, as soon as you re-supply the staging sign-in details. Nobody else needs to do anything.</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>1. Send me the staging username and password again (they are deliberately not stored in the repository, and this machine has been cleared).
-2. I sign in, seed two customers each with an "Approves Work" contact, raise an estimate for the first, and walk the five steps.
-3. I record Passed or Failed against this case and tell you the same day.
-Note: the case belongs to Vladimir Tomovic and is flagged Automated, so its wording will not be touched - only a result recorded.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="62" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
+    <row r="6" ht="62" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>NOTE on the two OBSOLETE tickets</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>SV-9804 and SV-9805 were raised for C44902 and C44907 and you closed them as OBSOLETE on 7 September. The cases are still blocked. Closing the tickets did not make the situations testable - it means no ticket is tracking them, so the decisions in this sheet are the only route.</t>
         </is>

</xml_diff>

<commit_message>
C44916: restate the block with Milan Zivanovic's ruling and the ticket link
Milan on SV-9710, 7 Sep: IBS has never worked on any environment except
production, and no sandbox account has ever been received. Combined with the
invoice redesign existing only on staging and not yet in production, the two never
overlap - so no environment today can show a real approval code on a redesigned
invoice. Not a mapping gap, and not a defect in the invoice work.

The run comment now carries the ticket link, Milan's words quoted in full, the
articulation, and the two routes that unblock it. Workbook row rewritten to match.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FWbxRKg4riKCp3gpbbwYzA
</commit_message>
<xml_diff>
--- a/build/invoice-ui-refresh/execution-2026-09-07/Invoice-UI-Refresh_Failed-and-Blocked-Cases_2026-09-08.xlsx
+++ b/build/invoice-ui-refresh/execution-2026-09-07/Invoice-UI-Refresh_Failed-and-Blocked-Cases_2026-09-08.xlsx
@@ -1239,12 +1239,12 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>KEEP - the case is good, only the environment is short</t>
+          <t>KEEP - good case, but it cannot be run anywhere yet</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>The case is fine. It checks that an approval code from the integrated billing service prints on the invoice. The problem is that this environment cannot request one of those approvals, so no approval code ever exists to print. Integrated billing IS switched on for the organisation - the remit-to payee and customer accounts are configured - but the approval request itself cannot be made here.</t>
+          <t>The case is fine. It checks that an approval code from the integrated billing service prints on the invoice. The problem is that the two things it needs are in different places and never meet. The invoice redesign this case tests exists ONLY on staging and has not been released to production yet. Integrated billing works ONLY in production - it has never worked on staging or on any QA branch. So there is nowhere today that a real approval code can appear on a redesigned invoice. On staging, integrated billing is not connected at all: no credentials, no base URL, and every shop location has an empty IBS Location ID, even though customers carry IBS account numbers.</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
@@ -1264,23 +1264,21 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Someone with access to the integrated billing service needs to do ONE of these:
-(A) Enable approval requests on this environment, or
-(B) Seed a single work order that already carries a real approval code, and send me its number.
-Option B is far quicker and is enough for the test.</t>
+          <t>Nothing from you right now, and no new ticket. Milan Zivanovic (development) has already ruled on SV-9710, 7 September 2026, in his own words: "IBS has never worked on any other env than production, just skip testing customers that have IBS number for now". He also asked Sasha Grosman for an IBS sandbox account: "we will need at some point that IBS sandbox/test account. We have never received it."</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>YOU, or whoever owns the integrated billing integration. The existing ticket SV-9710 is Open and assigned to Milomir Kotlajic. I cannot do this myself - it needs the billing service, not the app.</t>
+          <t>SASHA GROSMAN, if we want this tested before release - she is the one Milan asked for the IBS sandbox account. Otherwise nobody: it clears itself once the redesign reaches production.</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>1. Add a comment to SV-9710 asking: can a work order with a stored approval code be seeded on staging?
-2. When it exists, send me the work order number.
-3. I open it, click Finance, and check the document shows a field labelled exactly "Approval Code" carrying that code, and that the code no longer appears under the "Authorized By" area.
-4. I report the same day.</t>
+          <t>There are only two ways this case can ever run, whichever comes first:
+(A) Someone obtains an IBS sandbox or test account, connects it and maps the shop locations. Milan has already asked Sasha Grosman for this on SV-9710 and it has never been supplied. Chase that if you want the chip verified BEFORE release.
+(B) The invoice redesign is released to production, where integrated billing already works, and the case is run there afterwards.
+In the meantime follow Milan's instruction: skip testing customers that carry an IBS number.
+Be aware of the consequence: if we ship first, the Approval Code chip goes to production having never been tested. That is a known and accepted gap, not an oversight.</t>
         </is>
       </c>
     </row>

</xml_diff>